<commit_message>
Fix navigation losing the enumerator's place, and drop the auto-advance
Position was an index into shown[], which render() rebuilds from the
relevance rules every time. Answering a gate question changes that array's
length, so every index after it silently referred to a different question -
which in the field looks like typed answers disappearing. Position is now
tracked by question name.

The radio auto-advance is gone. It fired 120ms after any radio was touched,
so a question could not be revisited and corrected without being thrown
forward again, and the timer was never cancelled.

knows_monthly_income was a yes/no answering 'month by month, or one total?'.
Now a two-option choice; codes unchanged so downstream tests still hold.

Adds checks/07_navigation_test.js, which drives the form's real navigation
code headlessly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/replication/final_instrument/questionnaire/Kedarnath_final_kobo.xlsx
+++ b/replication/final_instrument/questionnaire/Kedarnath_final_kobo.xlsx
@@ -2538,7 +2538,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>select_one yn</t>
+          <t>select_one recall</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -8337,7 +8337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D266"/>
+  <dimension ref="A1:D268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11745,7 +11745,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>referral</t>
+          <t>recall</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -11753,32 +11753,32 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>A family member already working here</t>
+          <t>Month by month</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>यहाँ पहले से काम कर रहा घरवाला</t>
+          <t>हर महीने का अलग-अलग</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>referral</t>
+          <t>recall</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>A friend or someone from the village</t>
+          <t>One total for the whole year</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>दोस्त या गाँव का कोई आदमी</t>
+          <t>पूरे साल का एक जोड़</t>
         </is>
       </c>
     </row>
@@ -11789,16 +11789,16 @@
         </is>
       </c>
       <c r="B173" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>A thekedar or contractor I now work for</t>
+          <t>A family member already working here</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>ठेकेदार जिसके लिए मैं अब काम करता हूँ</t>
+          <t>यहाँ पहले से काम कर रहा घरवाला</t>
         </is>
       </c>
     </row>
@@ -11809,16 +11809,16 @@
         </is>
       </c>
       <c r="B174" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>An agent or middleman who placed me (usually for a fee)</t>
+          <t>A friend or someone from the village</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>एजेंट या बिचौलिया जिसने लगवाया (आम तौर पर पैसे लेकर)</t>
+          <t>दोस्त या गाँव का कोई आदमी</t>
         </is>
       </c>
     </row>
@@ -11829,16 +11829,16 @@
         </is>
       </c>
       <c r="B175" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>No one; I found it myself</t>
+          <t>A thekedar or contractor I now work for</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>कोई नहीं, ख़ुद ढूँढा</t>
+          <t>ठेकेदार जिसके लिए मैं अब काम करता हूँ</t>
         </is>
       </c>
     </row>
@@ -11849,16 +11849,16 @@
         </is>
       </c>
       <c r="B176" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>The employer called me directly</t>
+          <t>An agent or middleman who placed me (usually for a fee)</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>मालिक ने सीधे बुलाया</t>
+          <t>एजेंट या बिचौलिया जिसने लगवाया (आम तौर पर पैसे लेकर)</t>
         </is>
       </c>
     </row>
@@ -11869,56 +11869,56 @@
         </is>
       </c>
       <c r="B177" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Someone else</t>
+          <t>No one; I found it myself</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>कोई और</t>
+          <t>कोई नहीं, ख़ुद ढूँढा</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>remitmode</t>
+          <t>referral</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Bank transfer</t>
+          <t>The employer called me directly</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>बैंक से</t>
+          <t>मालिक ने सीधे बुलाया</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>remitmode</t>
+          <t>referral</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>UPI or phone payment</t>
+          <t>Someone else</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>UPI या फ़ोन से</t>
+          <t>कोई और</t>
         </is>
       </c>
     </row>
@@ -11929,16 +11929,16 @@
         </is>
       </c>
       <c r="B180" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Money order or post office</t>
+          <t>Bank transfer</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>मनीऑर्डर या डाकघर से</t>
+          <t>बैंक से</t>
         </is>
       </c>
     </row>
@@ -11949,16 +11949,16 @@
         </is>
       </c>
       <c r="B181" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Sent with someone going home</t>
+          <t>UPI or phone payment</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>घर जा रहे किसी के हाथ</t>
+          <t>UPI या फ़ोन से</t>
         </is>
       </c>
     </row>
@@ -11969,16 +11969,16 @@
         </is>
       </c>
       <c r="B182" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Carried it myself</t>
+          <t>Money order or post office</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>ख़ुद लेकर गए</t>
+          <t>मनीऑर्डर या डाकघर से</t>
         </is>
       </c>
     </row>
@@ -11989,56 +11989,56 @@
         </is>
       </c>
       <c r="B183" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Sent with someone going home</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>कोई और तरीक़ा</t>
+          <t>घर जा रहे किसी के हाथ</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>roof</t>
+          <t>remitmode</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Thatch/wood/mud</t>
+          <t>Carried it myself</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>फूस/लकड़ी/मिट्टी</t>
+          <t>ख़ुद लेकर गए</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>roof</t>
+          <t>remitmode</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Tin/GI sheet</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>टीन/चादर</t>
+          <t>कोई और तरीक़ा</t>
         </is>
       </c>
     </row>
@@ -12049,96 +12049,96 @@
         </is>
       </c>
       <c r="B186" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Concrete/RCC</t>
+          <t>Thatch/wood/mud</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>छत (कंक्रीट/RCC)</t>
+          <t>फूस/लकड़ी/मिट्टी</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>sex</t>
+          <t>roof</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Tin/GI sheet</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>पुरुष</t>
+          <t>टीन/चादर</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>sex</t>
+          <t>roof</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Concrete/RCC</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>महिला</t>
+          <t>छत (कंक्रीट/RCC)</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>stance</t>
+          <t>sex</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>पक्ष में</t>
+          <t>पुरुष</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>stance</t>
+          <t>sex</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>बीच में</t>
+          <t>महिला</t>
         </is>
       </c>
     </row>
@@ -12149,16 +12149,16 @@
         </is>
       </c>
       <c r="B191" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Oppose</t>
+          <t>Support</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>ख़िलाफ़</t>
+          <t>पक्ष में</t>
         </is>
       </c>
     </row>
@@ -12169,56 +12169,56 @@
         </is>
       </c>
       <c r="B192" t="n">
-        <v>98</v>
+        <v>2</v>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Don't know / prefer not to say</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>पता नहीं / बताना नहीं चाहते</t>
+          <t>बीच में</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>stance</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Andhra Pradesh</t>
+          <t>Oppose</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>आंध्र प्रदेश</t>
+          <t>ख़िलाफ़</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>stance</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>2</v>
+        <v>98</v>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Arunachal Pradesh</t>
+          <t>Don't know / prefer not to say</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>अरुणाचल प्रदेश</t>
+          <t>पता नहीं / बताना नहीं चाहते</t>
         </is>
       </c>
     </row>
@@ -12229,16 +12229,16 @@
         </is>
       </c>
       <c r="B195" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Assam</t>
+          <t>Andhra Pradesh</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>असम</t>
+          <t>आंध्र प्रदेश</t>
         </is>
       </c>
     </row>
@@ -12249,16 +12249,16 @@
         </is>
       </c>
       <c r="B196" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Bihar</t>
+          <t>Arunachal Pradesh</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>बिहार</t>
+          <t>अरुणाचल प्रदेश</t>
         </is>
       </c>
     </row>
@@ -12269,16 +12269,16 @@
         </is>
       </c>
       <c r="B197" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Chhattisgarh</t>
+          <t>Assam</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>छत्तीसगढ़</t>
+          <t>असम</t>
         </is>
       </c>
     </row>
@@ -12289,16 +12289,16 @@
         </is>
       </c>
       <c r="B198" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Goa</t>
+          <t>Bihar</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>गोवा</t>
+          <t>बिहार</t>
         </is>
       </c>
     </row>
@@ -12309,16 +12309,16 @@
         </is>
       </c>
       <c r="B199" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Gujarat</t>
+          <t>Chhattisgarh</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>गुजरात</t>
+          <t>छत्तीसगढ़</t>
         </is>
       </c>
     </row>
@@ -12329,16 +12329,16 @@
         </is>
       </c>
       <c r="B200" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Haryana</t>
+          <t>Goa</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>हरियाणा</t>
+          <t>गोवा</t>
         </is>
       </c>
     </row>
@@ -12349,16 +12349,16 @@
         </is>
       </c>
       <c r="B201" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Himachal Pradesh</t>
+          <t>Gujarat</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>हिमाचल प्रदेश</t>
+          <t>गुजरात</t>
         </is>
       </c>
     </row>
@@ -12369,16 +12369,16 @@
         </is>
       </c>
       <c r="B202" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Jharkhand</t>
+          <t>Haryana</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>झारखंड</t>
+          <t>हरियाणा</t>
         </is>
       </c>
     </row>
@@ -12389,16 +12389,16 @@
         </is>
       </c>
       <c r="B203" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Karnataka</t>
+          <t>Himachal Pradesh</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>कर्नाटक</t>
+          <t>हिमाचल प्रदेश</t>
         </is>
       </c>
     </row>
@@ -12409,16 +12409,16 @@
         </is>
       </c>
       <c r="B204" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Kerala</t>
+          <t>Jharkhand</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>केरल</t>
+          <t>झारखंड</t>
         </is>
       </c>
     </row>
@@ -12429,16 +12429,16 @@
         </is>
       </c>
       <c r="B205" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Madhya Pradesh</t>
+          <t>Karnataka</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>मध्य प्रदेश</t>
+          <t>कर्नाटक</t>
         </is>
       </c>
     </row>
@@ -12449,16 +12449,16 @@
         </is>
       </c>
       <c r="B206" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Maharashtra</t>
+          <t>Kerala</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>महाराष्ट्र</t>
+          <t>केरल</t>
         </is>
       </c>
     </row>
@@ -12469,16 +12469,16 @@
         </is>
       </c>
       <c r="B207" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Manipur</t>
+          <t>Madhya Pradesh</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>मणिपुर</t>
+          <t>मध्य प्रदेश</t>
         </is>
       </c>
     </row>
@@ -12489,16 +12489,16 @@
         </is>
       </c>
       <c r="B208" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Meghalaya</t>
+          <t>Maharashtra</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>मेघालय</t>
+          <t>महाराष्ट्र</t>
         </is>
       </c>
     </row>
@@ -12509,16 +12509,16 @@
         </is>
       </c>
       <c r="B209" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Mizoram</t>
+          <t>Manipur</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>मिज़ोरम</t>
+          <t>मणिपुर</t>
         </is>
       </c>
     </row>
@@ -12529,16 +12529,16 @@
         </is>
       </c>
       <c r="B210" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Nagaland</t>
+          <t>Meghalaya</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>नागालैंड</t>
+          <t>मेघालय</t>
         </is>
       </c>
     </row>
@@ -12549,16 +12549,16 @@
         </is>
       </c>
       <c r="B211" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Odisha</t>
+          <t>Mizoram</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>ओडिशा</t>
+          <t>मिज़ोरम</t>
         </is>
       </c>
     </row>
@@ -12569,16 +12569,16 @@
         </is>
       </c>
       <c r="B212" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Punjab</t>
+          <t>Nagaland</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>पंजाब</t>
+          <t>नागालैंड</t>
         </is>
       </c>
     </row>
@@ -12589,16 +12589,16 @@
         </is>
       </c>
       <c r="B213" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Rajasthan</t>
+          <t>Odisha</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>राजस्थान</t>
+          <t>ओडिशा</t>
         </is>
       </c>
     </row>
@@ -12609,16 +12609,16 @@
         </is>
       </c>
       <c r="B214" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Sikkim</t>
+          <t>Punjab</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>सिक्किम</t>
+          <t>पंजाब</t>
         </is>
       </c>
     </row>
@@ -12629,16 +12629,16 @@
         </is>
       </c>
       <c r="B215" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Tamil Nadu</t>
+          <t>Rajasthan</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>तमिलनाडु</t>
+          <t>राजस्थान</t>
         </is>
       </c>
     </row>
@@ -12649,16 +12649,16 @@
         </is>
       </c>
       <c r="B216" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Telangana</t>
+          <t>Sikkim</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>तेलंगाना</t>
+          <t>सिक्किम</t>
         </is>
       </c>
     </row>
@@ -12669,16 +12669,16 @@
         </is>
       </c>
       <c r="B217" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Tripura</t>
+          <t>Tamil Nadu</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>त्रिपुरा</t>
+          <t>तमिलनाडु</t>
         </is>
       </c>
     </row>
@@ -12689,16 +12689,16 @@
         </is>
       </c>
       <c r="B218" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Uttar Pradesh</t>
+          <t>Telangana</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>उत्तर प्रदेश</t>
+          <t>तेलंगाना</t>
         </is>
       </c>
     </row>
@@ -12709,16 +12709,16 @@
         </is>
       </c>
       <c r="B219" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Uttarakhand</t>
+          <t>Tripura</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>उत्तराखंड</t>
+          <t>त्रिपुरा</t>
         </is>
       </c>
     </row>
@@ -12729,16 +12729,16 @@
         </is>
       </c>
       <c r="B220" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>West Bengal</t>
+          <t>Uttar Pradesh</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>पश्चिम बंगाल</t>
+          <t>उत्तर प्रदेश</t>
         </is>
       </c>
     </row>
@@ -12749,16 +12749,16 @@
         </is>
       </c>
       <c r="B221" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Andaman and Nicobar Islands</t>
+          <t>Uttarakhand</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>अंडमान और निकोबार द्वीप समूह</t>
+          <t>उत्तराखंड</t>
         </is>
       </c>
     </row>
@@ -12769,16 +12769,16 @@
         </is>
       </c>
       <c r="B222" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Chandigarh</t>
+          <t>West Bengal</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>चंडीगढ़</t>
+          <t>पश्चिम बंगाल</t>
         </is>
       </c>
     </row>
@@ -12789,16 +12789,16 @@
         </is>
       </c>
       <c r="B223" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Dadra and Nagar Haveli and Daman and Diu</t>
+          <t>Andaman and Nicobar Islands</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>दादरा और नगर हवेली तथा दमन और दीव</t>
+          <t>अंडमान और निकोबार द्वीप समूह</t>
         </is>
       </c>
     </row>
@@ -12809,16 +12809,16 @@
         </is>
       </c>
       <c r="B224" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Chandigarh</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>दिल्ली</t>
+          <t>चंडीगढ़</t>
         </is>
       </c>
     </row>
@@ -12829,16 +12829,16 @@
         </is>
       </c>
       <c r="B225" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Jammu and Kashmir</t>
+          <t>Dadra and Nagar Haveli and Daman and Diu</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>जम्मू और कश्मीर</t>
+          <t>दादरा और नगर हवेली तथा दमन और दीव</t>
         </is>
       </c>
     </row>
@@ -12849,16 +12849,16 @@
         </is>
       </c>
       <c r="B226" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Ladakh</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>लद्दाख</t>
+          <t>दिल्ली</t>
         </is>
       </c>
     </row>
@@ -12869,16 +12869,16 @@
         </is>
       </c>
       <c r="B227" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Lakshadweep</t>
+          <t>Jammu and Kashmir</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>लक्षद्वीप</t>
+          <t>जम्मू और कश्मीर</t>
         </is>
       </c>
     </row>
@@ -12889,16 +12889,16 @@
         </is>
       </c>
       <c r="B228" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Puducherry</t>
+          <t>Ladakh</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>पुदुच्चेरी</t>
+          <t>लद्दाख</t>
         </is>
       </c>
     </row>
@@ -12909,56 +12909,56 @@
         </is>
       </c>
       <c r="B229" t="n">
-        <v>99</v>
+        <v>35</v>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Outside India</t>
+          <t>Lakshadweep</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>भारत से बाहर</t>
+          <t>लक्षद्वीप</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>task3</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B230" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Yes, regularly in my main Yatra work</t>
+          <t>Puducherry</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>हाँ, अपने मुख्य यात्रा-काम में नियमित</t>
+          <t>पुदुच्चेरी</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>task3</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B231" t="n">
-        <v>2</v>
+        <v>99</v>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Not in my main work, but done before elsewhere</t>
+          <t>Outside India</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>मुख्य काम में नहीं, पर पहले कहीं और किया है</t>
+          <t>भारत से बाहर</t>
         </is>
       </c>
     </row>
@@ -12969,56 +12969,56 @@
         </is>
       </c>
       <c r="B232" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Never done</t>
+          <t>Yes, regularly in my main Yatra work</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>कभी नहीं किया</t>
+          <t>हाँ, अपने मुख्य यात्रा-काम में नियमित</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>toilet</t>
+          <t>task3</t>
         </is>
       </c>
       <c r="B233" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>No toilet / open defecation</t>
+          <t>Not in my main work, but done before elsewhere</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>शौचालय नहीं / खुले में</t>
+          <t>मुख्य काम में नहीं, पर पहले कहीं और किया है</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>toilet</t>
+          <t>task3</t>
         </is>
       </c>
       <c r="B234" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Pit latrine without slab or open pit</t>
+          <t>Never done</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>बिना ढँके गड्ढे वाला शौचालय</t>
+          <t>कभी नहीं किया</t>
         </is>
       </c>
     </row>
@@ -13029,16 +13029,16 @@
         </is>
       </c>
       <c r="B235" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Improved toilet, but shared with other households</t>
+          <t>No toilet / open defecation</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>अच्छा शौचालय, पर दूसरे घरों के साथ साझा</t>
+          <t>शौचालय नहीं / खुले में</t>
         </is>
       </c>
     </row>
@@ -13049,56 +13049,56 @@
         </is>
       </c>
       <c r="B236" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Improved toilet, used only by this household</t>
+          <t>Pit latrine without slab or open pit</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>अच्छा शौचालय, सिर्फ़ इसी घर के लिए</t>
+          <t>बिना ढँके गड्ढे वाला शौचालय</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>trtype</t>
+          <t>toilet</t>
         </is>
       </c>
       <c r="B237" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>ITI or other trade course</t>
+          <t>Improved toilet, but shared with other households</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>ITI या कोई और कारीगरी का कोर्स</t>
+          <t>अच्छा शौचालय, पर दूसरे घरों के साथ साझा</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>trtype</t>
+          <t>toilet</t>
         </is>
       </c>
       <c r="B238" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Hotel, catering or tourism</t>
+          <t>Improved toilet, used only by this household</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>होटल, खानपान या पर्यटन</t>
+          <t>अच्छा शौचालय, सिर्फ़ इसी घर के लिए</t>
         </is>
       </c>
     </row>
@@ -13109,16 +13109,16 @@
         </is>
       </c>
       <c r="B239" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Driving</t>
+          <t>ITI or other trade course</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>गाड़ी चलाना</t>
+          <t>ITI या कोई और कारीगरी का कोर्स</t>
         </is>
       </c>
     </row>
@@ -13129,16 +13129,16 @@
         </is>
       </c>
       <c r="B240" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Mobile, computer or electrical repair</t>
+          <t>Hotel, catering or tourism</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>मोबाइल, कंप्यूटर या बिजली की मरम्मत</t>
+          <t>होटल, खानपान या पर्यटन</t>
         </is>
       </c>
     </row>
@@ -13149,16 +13149,16 @@
         </is>
       </c>
       <c r="B241" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Tailoring or handicraft</t>
+          <t>Driving</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>सिलाई या दस्तकारी</t>
+          <t>गाड़ी चलाना</t>
         </is>
       </c>
     </row>
@@ -13169,16 +13169,16 @@
         </is>
       </c>
       <c r="B242" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Animal handling or veterinary</t>
+          <t>Mobile, computer or electrical repair</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>जानवरों की देखभाल या पशु-चिकित्सा</t>
+          <t>मोबाइल, कंप्यूटर या बिजली की मरम्मत</t>
         </is>
       </c>
     </row>
@@ -13189,16 +13189,16 @@
         </is>
       </c>
       <c r="B243" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Construction trade (mason, carpenter, plumber)</t>
+          <t>Tailoring or handicraft</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>निर्माण का काम (राजमिस्त्री, बढ़ई, प्लंबर)</t>
+          <t>सिलाई या दस्तकारी</t>
         </is>
       </c>
     </row>
@@ -13209,16 +13209,16 @@
         </is>
       </c>
       <c r="B244" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Health or first aid</t>
+          <t>Animal handling or veterinary</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>सेहत या प्राथमिक उपचार</t>
+          <t>जानवरों की देखभाल या पशु-चिकित्सा</t>
         </is>
       </c>
     </row>
@@ -13229,56 +13229,56 @@
         </is>
       </c>
       <c r="B245" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Construction trade (mason, carpenter, plumber)</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>कोई और</t>
+          <t>निर्माण का काम (राजमिस्त्री, बढ़ई, प्लंबर)</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>trtype</t>
         </is>
       </c>
       <c r="B246" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Mud, thatch, bamboo or other natural material</t>
+          <t>Health or first aid</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>मिट्टी, फूस, बाँस या ऐसी ही कोई चीज़</t>
+          <t>सेहत या प्राथमिक उपचार</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>trtype</t>
         </is>
       </c>
       <c r="B247" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Unburnt brick, wood or tin</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>कच्ची ईंट, लकड़ी या टीन</t>
+          <t>कोई और</t>
         </is>
       </c>
     </row>
@@ -13289,56 +13289,56 @@
         </is>
       </c>
       <c r="B248" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Burnt brick, cement, concrete or stone</t>
+          <t>Mud, thatch, bamboo or other natural material</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>पक्की ईंट, सीमेंट, कंक्रीट या पत्थर</t>
+          <t>मिट्टी, फूस, बाँस या ऐसी ही कोई चीज़</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="B249" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Piped into the house or yard</t>
+          <t>Unburnt brick, wood or tin</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>घर या आँगन में नल</t>
+          <t>कच्ची ईंट, लकड़ी या टीन</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="B250" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Public tap or standpipe</t>
+          <t>Burnt brick, cement, concrete or stone</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>सार्वजनिक नल या स्टैंडपोस्ट</t>
+          <t>पक्की ईंट, सीमेंट, कंक्रीट या पत्थर</t>
         </is>
       </c>
     </row>
@@ -13349,16 +13349,16 @@
         </is>
       </c>
       <c r="B251" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Handpump, tubewell or borewell</t>
+          <t>Piped into the house or yard</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>हैंडपंप, ट्यूबवेल या बोरवेल</t>
+          <t>घर या आँगन में नल</t>
         </is>
       </c>
     </row>
@@ -13369,16 +13369,16 @@
         </is>
       </c>
       <c r="B252" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Protected well or protected spring</t>
+          <t>Public tap or standpipe</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>ढका हुआ कुआँ या ढका हुआ सोता</t>
+          <t>सार्वजनिक नल या स्टैंडपोस्ट</t>
         </is>
       </c>
     </row>
@@ -13389,16 +13389,16 @@
         </is>
       </c>
       <c r="B253" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Rainwater collection</t>
+          <t>Handpump, tubewell or borewell</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>बारिश का पानी जमा करके</t>
+          <t>हैंडपंप, ट्यूबवेल या बोरवेल</t>
         </is>
       </c>
     </row>
@@ -13409,16 +13409,16 @@
         </is>
       </c>
       <c r="B254" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Bottled, packaged or community RO</t>
+          <t>Protected well or protected spring</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>बोतलबंद, पैकेट या सामुदायिक RO</t>
+          <t>ढका हुआ कुआँ या ढका हुआ सोता</t>
         </is>
       </c>
     </row>
@@ -13429,16 +13429,16 @@
         </is>
       </c>
       <c r="B255" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Unprotected well or unprotected spring</t>
+          <t>Rainwater collection</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>खुला कुआँ या खुला सोता</t>
+          <t>बारिश का पानी जमा करके</t>
         </is>
       </c>
     </row>
@@ -13449,16 +13449,16 @@
         </is>
       </c>
       <c r="B256" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>River, stream, pond or canal</t>
+          <t>Bottled, packaged or community RO</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>नदी, गाड़, तालाब या नहर</t>
+          <t>बोतलबंद, पैकेट या सामुदायिक RO</t>
         </is>
       </c>
     </row>
@@ -13469,56 +13469,56 @@
         </is>
       </c>
       <c r="B257" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Tanker truck or cart with drum</t>
+          <t>Unprotected well or unprotected spring</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>टैंकर या ड्रम वाली गाड़ी</t>
+          <t>खुला कुआँ या खुला सोता</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>workins</t>
+          <t>water</t>
         </is>
       </c>
       <c r="B258" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Yes, through work</t>
+          <t>River, stream, pond or canal</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>हाँ, काम की तरफ़ से</t>
+          <t>नदी, गाड़, तालाब या नहर</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>workins</t>
+          <t>water</t>
         </is>
       </c>
       <c r="B259" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Only private or other insurance</t>
+          <t>Tanker truck or cart with drum</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>सिर्फ़ अपना या कोई और बीमा</t>
+          <t>टैंकर या ड्रम वाली गाड़ी</t>
         </is>
       </c>
     </row>
@@ -13529,16 +13529,16 @@
         </is>
       </c>
       <c r="B260" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Yes, through work</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>कोई नहीं</t>
+          <t>हाँ, काम की तरफ़ से</t>
         </is>
       </c>
     </row>
@@ -13549,63 +13549,63 @@
         </is>
       </c>
       <c r="B261" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Don't know</t>
+          <t>Only private or other insurance</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>पता नहीं</t>
+          <t>सिर्फ़ अपना या कोई और बीमा</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>yn</t>
+          <t>workins</t>
         </is>
       </c>
       <c r="B262" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>None</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>नहीं</t>
+          <t>कोई नहीं</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>yn</t>
+          <t>workins</t>
         </is>
       </c>
       <c r="B263" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Don't know</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>हाँ</t>
+          <t>पता नहीं</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>yndk</t>
+          <t>yn</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -13625,7 +13625,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>yndk</t>
+          <t>yn</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -13649,14 +13649,54 @@
         </is>
       </c>
       <c r="B266" t="n">
+        <v>0</v>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>नहीं</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>yndk</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>1</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>yndk</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
         <v>97</v>
       </c>
-      <c r="C266" t="inlineStr">
+      <c r="C268" t="inlineStr">
         <is>
           <t>Don't know</t>
         </is>
       </c>
-      <c r="D266" t="inlineStr">
+      <c r="D268" t="inlineStr">
         <is>
           <t>पता नहीं</t>
         </is>

</xml_diff>